<commit_message>
Adding cell lysate ELISAs
</commit_message>
<xml_diff>
--- a/analysis/plotting.xlsx
+++ b/analysis/plotting.xlsx
@@ -27,17 +27,15 @@
     <sheet name="Figure 3f" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Figure 5a" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="Figure 5b" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Figure 5c" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Figure 5d" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Figure 5e" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Figure 5f" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Supplemental 6" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Figure 5d" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Figure 5c" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Supplemental 6" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="146">
   <si>
     <t xml:space="preserve">NHP</t>
   </si>
@@ -435,13 +433,31 @@
     <t xml:space="preserve">VEGF</t>
   </si>
   <si>
+    <t xml:space="preserve">Antigen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Immunoglobulin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endpoint titer</t>
+  </si>
+  <si>
     <t xml:space="preserve">IgM</t>
   </si>
   <si>
     <t xml:space="preserve">IgG</t>
   </si>
   <si>
-    <t xml:space="preserve">Dilution</t>
+    <t xml:space="preserve">EBOV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUDV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BDBV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAFV</t>
   </si>
   <si>
     <t xml:space="preserve">PercentReduction</t>
@@ -456,10 +472,7 @@
     <t xml:space="preserve">28</t>
   </si>
   <si>
-    <t xml:space="preserve">EBOV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TAFV</t>
+    <t xml:space="preserve">Dilution</t>
   </si>
 </sst>
 </file>
@@ -20976,6 +20989,12 @@
       <c r="C1" t="s">
         <v>132</v>
       </c>
+      <c r="D1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -20984,7 +21003,13 @@
       <c r="B2" t="n">
         <v>0</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20995,7 +21020,13 @@
       <c r="B3" t="n">
         <v>5</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E3" t="n">
         <v>100</v>
       </c>
     </row>
@@ -21006,7 +21037,13 @@
       <c r="B4" t="n">
         <v>7</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E4" t="n">
         <v>300</v>
       </c>
     </row>
@@ -21017,7 +21054,13 @@
       <c r="B5" t="n">
         <v>10</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s">
+        <v>135</v>
+      </c>
+      <c r="E5" t="n">
         <v>12800</v>
       </c>
     </row>
@@ -21028,7 +21071,13 @@
       <c r="B6" t="n">
         <v>15</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E6" t="n">
         <v>6400</v>
       </c>
     </row>
@@ -21039,7 +21088,13 @@
       <c r="B7" t="n">
         <v>28</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" t="s">
+        <v>135</v>
+      </c>
+      <c r="E7" t="n">
         <v>1200</v>
       </c>
     </row>
@@ -21050,7 +21105,13 @@
       <c r="B8" t="n">
         <v>0</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" t="s">
+        <v>135</v>
+      </c>
+      <c r="E8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21061,7 +21122,13 @@
       <c r="B9" t="n">
         <v>5</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21072,7 +21139,13 @@
       <c r="B10" t="n">
         <v>7</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" t="n">
         <v>100</v>
       </c>
     </row>
@@ -21083,7 +21156,13 @@
       <c r="B11" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" t="s">
+        <v>135</v>
+      </c>
+      <c r="E11" t="n">
         <v>800</v>
       </c>
     </row>
@@ -21094,7 +21173,13 @@
       <c r="B12" t="n">
         <v>15</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" t="s">
+        <v>135</v>
+      </c>
+      <c r="E12" t="n">
         <v>3200</v>
       </c>
     </row>
@@ -21105,7 +21190,13 @@
       <c r="B13" t="n">
         <v>28</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" t="s">
+        <v>135</v>
+      </c>
+      <c r="E13" t="n">
         <v>800</v>
       </c>
     </row>
@@ -21116,7 +21207,13 @@
       <c r="B14" t="n">
         <v>0</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21127,7 +21224,13 @@
       <c r="B15" t="n">
         <v>5</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" t="s">
+        <v>135</v>
+      </c>
+      <c r="E15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21138,7 +21241,13 @@
       <c r="B16" t="n">
         <v>7</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" t="s">
+        <v>135</v>
+      </c>
+      <c r="E16" t="n">
         <v>200</v>
       </c>
     </row>
@@ -21149,7 +21258,13 @@
       <c r="B17" t="n">
         <v>10</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" t="s">
+        <v>135</v>
+      </c>
+      <c r="E17" t="n">
         <v>1600</v>
       </c>
     </row>
@@ -21160,7 +21275,13 @@
       <c r="B18" t="n">
         <v>15</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>135</v>
+      </c>
+      <c r="E18" t="n">
         <v>2400</v>
       </c>
     </row>
@@ -21171,7 +21292,13 @@
       <c r="B19" t="n">
         <v>28</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" t="s">
+        <v>135</v>
+      </c>
+      <c r="E19" t="n">
         <v>400</v>
       </c>
     </row>
@@ -21182,7 +21309,13 @@
       <c r="B20" t="n">
         <v>0</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" t="s">
+        <v>135</v>
+      </c>
+      <c r="E20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21193,7 +21326,13 @@
       <c r="B21" t="n">
         <v>5</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" t="s">
+        <v>135</v>
+      </c>
+      <c r="E21" t="n">
         <v>200</v>
       </c>
     </row>
@@ -21204,7 +21343,13 @@
       <c r="B22" t="n">
         <v>7</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" t="s">
+        <v>135</v>
+      </c>
+      <c r="E22" t="n">
         <v>400</v>
       </c>
     </row>
@@ -21215,7 +21360,13 @@
       <c r="B23" t="n">
         <v>10</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" t="s">
+        <v>135</v>
+      </c>
+      <c r="E23" t="n">
         <v>800</v>
       </c>
     </row>
@@ -21226,7 +21377,13 @@
       <c r="B24" t="n">
         <v>15</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" t="s">
+        <v>135</v>
+      </c>
+      <c r="E24" t="n">
         <v>6400</v>
       </c>
     </row>
@@ -21237,7 +21394,13 @@
       <c r="B25" t="n">
         <v>28</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" t="s">
+        <v>135</v>
+      </c>
+      <c r="E25" t="n">
         <v>1600</v>
       </c>
     </row>
@@ -21260,7 +21423,13 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D1" t="s">
         <v>133</v>
+      </c>
+      <c r="E1" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="2">
@@ -21270,7 +21439,13 @@
       <c r="B2" t="n">
         <v>0</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21281,7 +21456,13 @@
       <c r="B3" t="n">
         <v>5</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21292,7 +21473,13 @@
       <c r="B4" t="n">
         <v>7</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E4" t="n">
         <v>200</v>
       </c>
     </row>
@@ -21303,7 +21490,13 @@
       <c r="B5" t="n">
         <v>10</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E5" t="n">
         <v>2400</v>
       </c>
     </row>
@@ -21314,7 +21507,13 @@
       <c r="B6" t="n">
         <v>15</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E6" t="n">
         <v>25600</v>
       </c>
     </row>
@@ -21325,7 +21524,13 @@
       <c r="B7" t="n">
         <v>28</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" t="s">
+        <v>136</v>
+      </c>
+      <c r="E7" t="n">
         <v>25600</v>
       </c>
     </row>
@@ -21336,7 +21541,13 @@
       <c r="B8" t="n">
         <v>0</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" t="s">
+        <v>136</v>
+      </c>
+      <c r="E8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21347,7 +21558,13 @@
       <c r="B9" t="n">
         <v>5</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>136</v>
+      </c>
+      <c r="E9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21358,7 +21575,13 @@
       <c r="B10" t="n">
         <v>7</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" t="s">
+        <v>136</v>
+      </c>
+      <c r="E10" t="n">
         <v>200</v>
       </c>
     </row>
@@ -21369,7 +21592,13 @@
       <c r="B11" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" t="s">
+        <v>136</v>
+      </c>
+      <c r="E11" t="n">
         <v>1600</v>
       </c>
     </row>
@@ -21380,7 +21609,13 @@
       <c r="B12" t="n">
         <v>15</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E12" t="n">
         <v>12800</v>
       </c>
     </row>
@@ -21391,7 +21626,13 @@
       <c r="B13" t="n">
         <v>28</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" t="s">
+        <v>136</v>
+      </c>
+      <c r="E13" t="n">
         <v>6400</v>
       </c>
     </row>
@@ -21402,7 +21643,13 @@
       <c r="B14" t="n">
         <v>0</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21413,7 +21660,13 @@
       <c r="B15" t="n">
         <v>5</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" t="s">
+        <v>136</v>
+      </c>
+      <c r="E15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21424,7 +21677,13 @@
       <c r="B16" t="n">
         <v>7</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" t="s">
+        <v>136</v>
+      </c>
+      <c r="E16" t="n">
         <v>200</v>
       </c>
     </row>
@@ -21435,7 +21694,13 @@
       <c r="B17" t="n">
         <v>10</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" t="s">
+        <v>136</v>
+      </c>
+      <c r="E17" t="n">
         <v>400</v>
       </c>
     </row>
@@ -21446,7 +21711,13 @@
       <c r="B18" t="n">
         <v>15</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>136</v>
+      </c>
+      <c r="E18" t="n">
         <v>3200</v>
       </c>
     </row>
@@ -21457,7 +21728,13 @@
       <c r="B19" t="n">
         <v>28</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" t="s">
+        <v>136</v>
+      </c>
+      <c r="E19" t="n">
         <v>3200</v>
       </c>
     </row>
@@ -21468,7 +21745,13 @@
       <c r="B20" t="n">
         <v>0</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" t="s">
+        <v>136</v>
+      </c>
+      <c r="E20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21479,7 +21762,13 @@
       <c r="B21" t="n">
         <v>5</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" t="s">
+        <v>136</v>
+      </c>
+      <c r="E21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21490,7 +21779,13 @@
       <c r="B22" t="n">
         <v>7</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" t="s">
+        <v>136</v>
+      </c>
+      <c r="E22" t="n">
         <v>100</v>
       </c>
     </row>
@@ -21501,7 +21796,13 @@
       <c r="B23" t="n">
         <v>10</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" t="s">
+        <v>136</v>
+      </c>
+      <c r="E23" t="n">
         <v>200</v>
       </c>
     </row>
@@ -21512,7 +21813,13 @@
       <c r="B24" t="n">
         <v>15</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" t="n">
         <v>3200</v>
       </c>
     </row>
@@ -21523,7 +21830,13 @@
       <c r="B25" t="n">
         <v>28</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" t="s">
+        <v>136</v>
+      </c>
+      <c r="E25" t="n">
         <v>1600</v>
       </c>
     </row>
@@ -21540,145 +21853,563 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1" t="s">
         <v>134</v>
-      </c>
-      <c r="C1" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" t="s">
         <v>136</v>
       </c>
-      <c r="B2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.4725274725275</v>
+      <c r="E2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
         <v>137</v>
       </c>
-      <c r="B3" t="n">
-        <v>10</v>
-      </c>
-      <c r="C3" t="n">
-        <v>51.8681318681319</v>
+      <c r="D3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
         <v>137</v>
       </c>
-      <c r="B4" t="n">
-        <v>20</v>
-      </c>
-      <c r="C4" t="n">
-        <v>30.1098901098901</v>
+      <c r="D4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
         <v>137</v>
       </c>
-      <c r="B5" t="n">
-        <v>40</v>
-      </c>
-      <c r="C5" t="n">
-        <v>22.1978021978022</v>
+      <c r="D5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" t="n">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
         <v>137</v>
       </c>
-      <c r="B6" t="n">
-        <v>80</v>
-      </c>
-      <c r="C6" t="n">
-        <v>19.5604395604396</v>
+      <c r="D6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E6" t="n">
+        <v>800</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" t="n">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
         <v>137</v>
       </c>
-      <c r="B7" t="n">
-        <v>160</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1.75824175824175</v>
+      <c r="D7" t="s">
+        <v>136</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1600</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>138</v>
+        <v>52</v>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
-      </c>
-      <c r="C8" t="n">
-        <v>84.8351648351648</v>
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D8" t="s">
+        <v>136</v>
+      </c>
+      <c r="E8" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>138</v>
+        <v>53</v>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
-      </c>
-      <c r="C9" t="n">
-        <v>74.9450549450549</v>
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D9" t="s">
+        <v>136</v>
+      </c>
+      <c r="E9" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="s">
         <v>138</v>
       </c>
-      <c r="B10" t="n">
-        <v>40</v>
-      </c>
-      <c r="C10" t="n">
-        <v>67.032967032967</v>
+      <c r="D10" t="s">
+        <v>136</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="s">
         <v>138</v>
       </c>
-      <c r="B11" t="n">
-        <v>80</v>
-      </c>
-      <c r="C11" t="n">
-        <v>48.5714285714286</v>
+      <c r="D11" t="s">
+        <v>136</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
         <v>138</v>
       </c>
-      <c r="B12" t="n">
-        <v>160</v>
-      </c>
-      <c r="C12" t="n">
-        <v>32.7472527472527</v>
+      <c r="D12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="s">
         <v>138</v>
       </c>
-      <c r="B13" t="n">
-        <v>320</v>
-      </c>
-      <c r="C13" t="n">
-        <v>18.9010989010989</v>
+      <c r="D13" t="s">
+        <v>136</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" t="n">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>138</v>
+      </c>
+      <c r="D14" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="n">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>138</v>
+      </c>
+      <c r="D15" t="s">
+        <v>136</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" t="n">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>138</v>
+      </c>
+      <c r="D16" t="s">
+        <v>136</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" t="n">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>138</v>
+      </c>
+      <c r="D17" t="s">
+        <v>136</v>
+      </c>
+      <c r="E17" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D18" t="s">
+        <v>136</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="s">
+        <v>139</v>
+      </c>
+      <c r="D19" t="s">
+        <v>136</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>139</v>
+      </c>
+      <c r="D20" t="s">
+        <v>136</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="s">
+        <v>139</v>
+      </c>
+      <c r="D21" t="s">
+        <v>136</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" t="n">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>139</v>
+      </c>
+      <c r="D22" t="s">
+        <v>136</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" t="n">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>139</v>
+      </c>
+      <c r="D23" t="s">
+        <v>136</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" t="n">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>139</v>
+      </c>
+      <c r="D24" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" t="n">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" t="s">
+        <v>136</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" t="s">
+        <v>140</v>
+      </c>
+      <c r="D26" t="s">
+        <v>136</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="s">
+        <v>140</v>
+      </c>
+      <c r="D27" t="s">
+        <v>136</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>140</v>
+      </c>
+      <c r="D28" t="s">
+        <v>136</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" t="s">
+        <v>140</v>
+      </c>
+      <c r="D29" t="s">
+        <v>136</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" t="n">
+        <v>28</v>
+      </c>
+      <c r="C30" t="s">
+        <v>140</v>
+      </c>
+      <c r="D30" t="s">
+        <v>136</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" t="n">
+        <v>28</v>
+      </c>
+      <c r="C31" t="s">
+        <v>140</v>
+      </c>
+      <c r="D31" t="s">
+        <v>136</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" t="n">
+        <v>28</v>
+      </c>
+      <c r="C32" t="s">
+        <v>140</v>
+      </c>
+      <c r="D32" t="s">
+        <v>136</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" t="n">
+        <v>28</v>
+      </c>
+      <c r="C33" t="s">
+        <v>140</v>
+      </c>
+      <c r="D33" t="s">
+        <v>136</v>
+      </c>
+      <c r="E33" t="n">
+        <v>800</v>
       </c>
     </row>
   </sheetData>
@@ -21694,156 +22425,145 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>134</v>
-      </c>
       <c r="C1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B2" t="n">
-        <v>10</v>
+        <v>49</v>
+      </c>
+      <c r="B2" t="s">
+        <v>142</v>
       </c>
       <c r="C2" t="n">
-        <v>24.8351648351648</v>
+        <v>27.4725274725275</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B3" t="n">
-        <v>10</v>
+        <v>49</v>
+      </c>
+      <c r="B3" t="s">
+        <v>143</v>
       </c>
       <c r="C3" t="n">
-        <v>71.6483516483516</v>
+        <v>51.8681318681319</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B4" t="n">
-        <v>20</v>
+        <v>49</v>
+      </c>
+      <c r="B4" t="s">
+        <v>144</v>
       </c>
       <c r="C4" t="n">
-        <v>66.3736263736264</v>
+        <v>84.8351648351648</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B5" t="n">
-        <v>40</v>
+        <v>51</v>
+      </c>
+      <c r="B5" t="s">
+        <v>142</v>
       </c>
       <c r="C5" t="n">
-        <v>55.8241758241758</v>
+        <v>24.8351648351648</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B6" t="n">
-        <v>80</v>
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>143</v>
       </c>
       <c r="C6" t="n">
-        <v>21.5384615384615</v>
+        <v>71.6483516483516</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B7" t="n">
-        <v>160</v>
+        <v>51</v>
+      </c>
+      <c r="B7" t="s">
+        <v>144</v>
       </c>
       <c r="C7" t="n">
-        <v>16.9230769230769</v>
+        <v>88.7912087912088</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B8" t="n">
-        <v>320</v>
+        <v>52</v>
+      </c>
+      <c r="B8" t="s">
+        <v>142</v>
       </c>
       <c r="C8" t="n">
-        <v>11.6483516483516</v>
+        <v>18.9010989010989</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>138</v>
-      </c>
-      <c r="B9" t="n">
-        <v>10</v>
+        <v>52</v>
+      </c>
+      <c r="B9" t="s">
+        <v>143</v>
       </c>
       <c r="C9" t="n">
-        <v>88.7912087912088</v>
+        <v>55.1648351648352</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>138</v>
-      </c>
-      <c r="B10" t="n">
-        <v>20</v>
+        <v>52</v>
+      </c>
+      <c r="B10" t="s">
+        <v>144</v>
       </c>
       <c r="C10" t="n">
-        <v>74.9450549450549</v>
+        <v>79.5604395604396</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>138</v>
-      </c>
-      <c r="B11" t="n">
-        <v>40</v>
+        <v>53</v>
+      </c>
+      <c r="B11" t="s">
+        <v>142</v>
       </c>
       <c r="C11" t="n">
-        <v>68.3516483516484</v>
+        <v>32.0879120879121</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>138</v>
-      </c>
-      <c r="B12" t="n">
-        <v>80</v>
+        <v>53</v>
+      </c>
+      <c r="B12" t="s">
+        <v>143</v>
       </c>
       <c r="C12" t="n">
-        <v>36.043956043956</v>
+        <v>49.2307692307692</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>138</v>
-      </c>
-      <c r="B13" t="n">
-        <v>160</v>
+        <v>53</v>
+      </c>
+      <c r="B13" t="s">
+        <v>144</v>
       </c>
       <c r="C13" t="n">
-        <v>30.7692307692308</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>138</v>
-      </c>
-      <c r="B14" t="n">
-        <v>320</v>
-      </c>
-      <c r="C14" t="n">
-        <v>20.2197802197802</v>
+        <v>82.1978021978022</v>
       </c>
     </row>
   </sheetData>
@@ -21859,347 +22579,6 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C2" t="n">
-        <v>18.9010989010989</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B3" t="n">
-        <v>10</v>
-      </c>
-      <c r="C3" t="n">
-        <v>55.1648351648352</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B4" t="n">
-        <v>20</v>
-      </c>
-      <c r="C4" t="n">
-        <v>43.2967032967033</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B5" t="n">
-        <v>40</v>
-      </c>
-      <c r="C5" t="n">
-        <v>33.4065934065934</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B6" t="n">
-        <v>80</v>
-      </c>
-      <c r="C6" t="n">
-        <v>26.1538461538461</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B7" t="n">
-        <v>160</v>
-      </c>
-      <c r="C7" t="n">
-        <v>23.5164835164835</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B8" t="n">
-        <v>320</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15.6043956043956</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>138</v>
-      </c>
-      <c r="B9" t="n">
-        <v>10</v>
-      </c>
-      <c r="C9" t="n">
-        <v>79.5604395604396</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>138</v>
-      </c>
-      <c r="B10" t="n">
-        <v>20</v>
-      </c>
-      <c r="C10" t="n">
-        <v>59.1208791208791</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>138</v>
-      </c>
-      <c r="B11" t="n">
-        <v>40</v>
-      </c>
-      <c r="C11" t="n">
-        <v>59.7802197802198</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>138</v>
-      </c>
-      <c r="B12" t="n">
-        <v>80</v>
-      </c>
-      <c r="C12" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>138</v>
-      </c>
-      <c r="B13" t="n">
-        <v>160</v>
-      </c>
-      <c r="C13" t="n">
-        <v>26.1538461538461</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>138</v>
-      </c>
-      <c r="B14" t="n">
-        <v>320</v>
-      </c>
-      <c r="C14" t="n">
-        <v>22.1978021978022</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C2" t="n">
-        <v>32.0879120879121</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B3" t="n">
-        <v>10</v>
-      </c>
-      <c r="C3" t="n">
-        <v>49.2307692307692</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B4" t="n">
-        <v>20</v>
-      </c>
-      <c r="C4" t="n">
-        <v>43.2967032967033</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B5" t="n">
-        <v>40</v>
-      </c>
-      <c r="C5" t="n">
-        <v>38.021978021978</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B6" t="n">
-        <v>80</v>
-      </c>
-      <c r="C6" t="n">
-        <v>28.7912087912088</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B7" t="n">
-        <v>160</v>
-      </c>
-      <c r="C7" t="n">
-        <v>13.6263736263736</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B8" t="n">
-        <v>320</v>
-      </c>
-      <c r="C8" t="n">
-        <v>12.967032967033</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>138</v>
-      </c>
-      <c r="B9" t="n">
-        <v>10</v>
-      </c>
-      <c r="C9" t="n">
-        <v>82.1978021978022</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>138</v>
-      </c>
-      <c r="B10" t="n">
-        <v>20</v>
-      </c>
-      <c r="C10" t="n">
-        <v>69.6703296703297</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>138</v>
-      </c>
-      <c r="B11" t="n">
-        <v>40</v>
-      </c>
-      <c r="C11" t="n">
-        <v>54.5054945054945</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>138</v>
-      </c>
-      <c r="B12" t="n">
-        <v>80</v>
-      </c>
-      <c r="C12" t="n">
-        <v>44.6153846153846</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>138</v>
-      </c>
-      <c r="B13" t="n">
-        <v>160</v>
-      </c>
-      <c r="C13" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>138</v>
-      </c>
-      <c r="B14" t="n">
-        <v>320</v>
-      </c>
-      <c r="C14" t="n">
-        <v>34.7252747252747</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>138</v>
-      </c>
-      <c r="B15" t="n">
-        <v>640</v>
-      </c>
-      <c r="C15" t="n">
-        <v>19.5604395604396</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -22209,10 +22588,10 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="E1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2">
@@ -22220,16 +22599,16 @@
         <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C2" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D2" t="n">
         <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>9.2274678111588</v>
+        <v>27.4725274725275</v>
       </c>
     </row>
     <row r="3">
@@ -22237,16 +22616,16 @@
         <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D3" t="n">
         <v>10</v>
       </c>
       <c r="E3" t="n">
-        <v>10.0463678516229</v>
+        <v>9.2274678111588</v>
       </c>
     </row>
     <row r="4">
@@ -22254,16 +22633,16 @@
         <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D4" t="n">
         <v>10</v>
       </c>
       <c r="E4" t="n">
-        <v>20.8154506437768</v>
+        <v>10.0463678516229</v>
       </c>
     </row>
     <row r="5">
@@ -22271,16 +22650,16 @@
         <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C5" t="s">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="D5" t="n">
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>20.7109737248841</v>
+        <v>51.8681318681319</v>
       </c>
     </row>
     <row r="6">
@@ -22288,16 +22667,16 @@
         <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C6" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E6" t="n">
-        <v>51.7167381974249</v>
+        <v>30.1098901098901</v>
       </c>
     </row>
     <row r="7">
@@ -22305,16 +22684,16 @@
         <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C7" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D7" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E7" t="n">
-        <v>38.1974248927039</v>
+        <v>22.1978021978022</v>
       </c>
     </row>
     <row r="8">
@@ -22322,16 +22701,16 @@
         <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C8" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D8" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="E8" t="n">
-        <v>25.3218884120172</v>
+        <v>19.5604395604396</v>
       </c>
     </row>
     <row r="9">
@@ -22339,16 +22718,16 @@
         <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C9" t="s">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>160</v>
       </c>
       <c r="E9" t="n">
-        <v>57.8052550231839</v>
+        <v>1.75824175824175</v>
       </c>
     </row>
     <row r="10">
@@ -22356,262 +22735,262 @@
         <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C10" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D10" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>22.5656877897991</v>
+        <v>20.8154506437768</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D11" t="n">
         <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>13.0901287553648</v>
+        <v>20.7109737248841</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C12" t="s">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="D12" t="n">
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>84.8351648351648</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D13" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E13" t="n">
-        <v>10.5150214592275</v>
+        <v>74.9450549450549</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B14" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C14" t="s">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E14" t="n">
-        <v>24.8840803709428</v>
+        <v>67.032967032967</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B15" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C15" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D15" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="E15" t="n">
-        <v>25.9656652360515</v>
+        <v>48.5714285714286</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B16" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C16" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D16" t="n">
-        <v>20</v>
+        <v>160</v>
       </c>
       <c r="E16" t="n">
-        <v>7.93991416309014</v>
+        <v>32.7472527472527</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C17" t="s">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="D17" t="n">
-        <v>10</v>
+        <v>320</v>
       </c>
       <c r="E17" t="n">
-        <v>18.8562596599691</v>
+        <v>18.9010989010989</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B18" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C18" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D18" t="n">
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>51.7167381974249</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B19" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C19" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D19" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E19" t="n">
-        <v>4.94590417310664</v>
+        <v>38.1974248927039</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B20" t="s">
+        <v>144</v>
+      </c>
+      <c r="C20" t="s">
         <v>137</v>
       </c>
-      <c r="C20" t="s">
-        <v>139</v>
-      </c>
       <c r="D20" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E20" t="n">
-        <v>42.7038626609442</v>
+        <v>25.3218884120172</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B21" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C21" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D21" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>14.3776824034335</v>
+        <v>57.8052550231839</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B22" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C22" t="s">
         <v>140</v>
       </c>
       <c r="D22" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E22" t="n">
-        <v>19.3199381761978</v>
+        <v>22.5656877897991</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B23" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C23" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D23" t="n">
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>34.3347639484979</v>
+        <v>24.8351648351648</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B24" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C24" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D24" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>11.1587982832618</v>
+        <v>13.0901287553648</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C25" t="s">
         <v>140</v>
@@ -22620,134 +22999,134 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>46.676970633694</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B26" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C26" t="s">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="D26" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>21.6383307573416</v>
+        <v>71.6483516483516</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C27" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E27" t="n">
-        <v>17.5965665236052</v>
+        <v>66.3736263736264</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B28" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C28" t="s">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="D28" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E28" t="n">
-        <v>11.9010819165379</v>
+        <v>55.8241758241758</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B29" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C29" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D29" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>21.5384615384615</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B30" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C30" t="s">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="D30" t="n">
-        <v>10</v>
+        <v>160</v>
       </c>
       <c r="E30" t="n">
-        <v>34.1576506955178</v>
+        <v>16.9230769230769</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B31" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C31" t="s">
-        <v>139</v>
+        <v>50</v>
       </c>
       <c r="D31" t="n">
-        <v>10</v>
+        <v>320</v>
       </c>
       <c r="E31" t="n">
-        <v>25.3218884120172</v>
+        <v>11.6483516483516</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B32" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C32" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D32" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>12.4463519313305</v>
+        <v>10.5150214592275</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B33" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C33" t="s">
         <v>140</v>
@@ -22756,6 +23135,890 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
+        <v>24.8840803709428</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>51</v>
+      </c>
+      <c r="B34" t="s">
+        <v>144</v>
+      </c>
+      <c r="C34" t="s">
+        <v>50</v>
+      </c>
+      <c r="D34" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" t="n">
+        <v>88.7912087912088</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" t="s">
+        <v>144</v>
+      </c>
+      <c r="C35" t="s">
+        <v>50</v>
+      </c>
+      <c r="D35" t="n">
+        <v>20</v>
+      </c>
+      <c r="E35" t="n">
+        <v>74.9450549450549</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>51</v>
+      </c>
+      <c r="B36" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D36" t="n">
+        <v>40</v>
+      </c>
+      <c r="E36" t="n">
+        <v>68.3516483516484</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" t="s">
+        <v>144</v>
+      </c>
+      <c r="C37" t="s">
+        <v>50</v>
+      </c>
+      <c r="D37" t="n">
+        <v>80</v>
+      </c>
+      <c r="E37" t="n">
+        <v>36.043956043956</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" t="s">
+        <v>144</v>
+      </c>
+      <c r="C38" t="s">
+        <v>50</v>
+      </c>
+      <c r="D38" t="n">
+        <v>160</v>
+      </c>
+      <c r="E38" t="n">
+        <v>30.7692307692308</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>51</v>
+      </c>
+      <c r="B39" t="s">
+        <v>144</v>
+      </c>
+      <c r="C39" t="s">
+        <v>50</v>
+      </c>
+      <c r="D39" t="n">
+        <v>320</v>
+      </c>
+      <c r="E39" t="n">
+        <v>20.2197802197802</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" t="s">
+        <v>144</v>
+      </c>
+      <c r="C40" t="s">
+        <v>137</v>
+      </c>
+      <c r="D40" t="n">
+        <v>10</v>
+      </c>
+      <c r="E40" t="n">
+        <v>25.9656652360515</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" t="s">
+        <v>144</v>
+      </c>
+      <c r="C41" t="s">
+        <v>137</v>
+      </c>
+      <c r="D41" t="n">
+        <v>20</v>
+      </c>
+      <c r="E41" t="n">
+        <v>7.93991416309014</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" t="s">
+        <v>144</v>
+      </c>
+      <c r="C42" t="s">
+        <v>140</v>
+      </c>
+      <c r="D42" t="n">
+        <v>10</v>
+      </c>
+      <c r="E42" t="n">
+        <v>18.8562596599691</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>52</v>
+      </c>
+      <c r="B43" t="s">
+        <v>142</v>
+      </c>
+      <c r="C43" t="s">
+        <v>50</v>
+      </c>
+      <c r="D43" t="n">
+        <v>10</v>
+      </c>
+      <c r="E43" t="n">
+        <v>18.9010989010989</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>52</v>
+      </c>
+      <c r="B44" t="s">
+        <v>142</v>
+      </c>
+      <c r="C44" t="s">
+        <v>137</v>
+      </c>
+      <c r="D44" t="n">
+        <v>10</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45" t="s">
+        <v>142</v>
+      </c>
+      <c r="C45" t="s">
+        <v>140</v>
+      </c>
+      <c r="D45" t="n">
+        <v>10</v>
+      </c>
+      <c r="E45" t="n">
+        <v>4.94590417310664</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>52</v>
+      </c>
+      <c r="B46" t="s">
+        <v>143</v>
+      </c>
+      <c r="C46" t="s">
+        <v>50</v>
+      </c>
+      <c r="D46" t="n">
+        <v>10</v>
+      </c>
+      <c r="E46" t="n">
+        <v>55.1648351648352</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>52</v>
+      </c>
+      <c r="B47" t="s">
+        <v>143</v>
+      </c>
+      <c r="C47" t="s">
+        <v>50</v>
+      </c>
+      <c r="D47" t="n">
+        <v>20</v>
+      </c>
+      <c r="E47" t="n">
+        <v>43.2967032967033</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>52</v>
+      </c>
+      <c r="B48" t="s">
+        <v>143</v>
+      </c>
+      <c r="C48" t="s">
+        <v>50</v>
+      </c>
+      <c r="D48" t="n">
+        <v>40</v>
+      </c>
+      <c r="E48" t="n">
+        <v>33.4065934065934</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B49" t="s">
+        <v>143</v>
+      </c>
+      <c r="C49" t="s">
+        <v>50</v>
+      </c>
+      <c r="D49" t="n">
+        <v>80</v>
+      </c>
+      <c r="E49" t="n">
+        <v>26.1538461538461</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" t="s">
+        <v>143</v>
+      </c>
+      <c r="C50" t="s">
+        <v>50</v>
+      </c>
+      <c r="D50" t="n">
+        <v>160</v>
+      </c>
+      <c r="E50" t="n">
+        <v>23.5164835164835</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51" t="s">
+        <v>143</v>
+      </c>
+      <c r="C51" t="s">
+        <v>50</v>
+      </c>
+      <c r="D51" t="n">
+        <v>320</v>
+      </c>
+      <c r="E51" t="n">
+        <v>15.6043956043956</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" t="s">
+        <v>143</v>
+      </c>
+      <c r="C52" t="s">
+        <v>137</v>
+      </c>
+      <c r="D52" t="n">
+        <v>10</v>
+      </c>
+      <c r="E52" t="n">
+        <v>42.7038626609442</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>143</v>
+      </c>
+      <c r="C53" t="s">
+        <v>137</v>
+      </c>
+      <c r="D53" t="n">
+        <v>20</v>
+      </c>
+      <c r="E53" t="n">
+        <v>14.3776824034335</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>52</v>
+      </c>
+      <c r="B54" t="s">
+        <v>143</v>
+      </c>
+      <c r="C54" t="s">
+        <v>140</v>
+      </c>
+      <c r="D54" t="n">
+        <v>10</v>
+      </c>
+      <c r="E54" t="n">
+        <v>19.3199381761978</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>52</v>
+      </c>
+      <c r="B55" t="s">
+        <v>144</v>
+      </c>
+      <c r="C55" t="s">
+        <v>50</v>
+      </c>
+      <c r="D55" t="n">
+        <v>10</v>
+      </c>
+      <c r="E55" t="n">
+        <v>79.5604395604396</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>52</v>
+      </c>
+      <c r="B56" t="s">
+        <v>144</v>
+      </c>
+      <c r="C56" t="s">
+        <v>50</v>
+      </c>
+      <c r="D56" t="n">
+        <v>20</v>
+      </c>
+      <c r="E56" t="n">
+        <v>59.1208791208791</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>52</v>
+      </c>
+      <c r="B57" t="s">
+        <v>144</v>
+      </c>
+      <c r="C57" t="s">
+        <v>50</v>
+      </c>
+      <c r="D57" t="n">
+        <v>40</v>
+      </c>
+      <c r="E57" t="n">
+        <v>59.7802197802198</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>52</v>
+      </c>
+      <c r="B58" t="s">
+        <v>144</v>
+      </c>
+      <c r="C58" t="s">
+        <v>50</v>
+      </c>
+      <c r="D58" t="n">
+        <v>80</v>
+      </c>
+      <c r="E58" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>52</v>
+      </c>
+      <c r="B59" t="s">
+        <v>144</v>
+      </c>
+      <c r="C59" t="s">
+        <v>50</v>
+      </c>
+      <c r="D59" t="n">
+        <v>160</v>
+      </c>
+      <c r="E59" t="n">
+        <v>26.1538461538461</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>52</v>
+      </c>
+      <c r="B60" t="s">
+        <v>144</v>
+      </c>
+      <c r="C60" t="s">
+        <v>50</v>
+      </c>
+      <c r="D60" t="n">
+        <v>320</v>
+      </c>
+      <c r="E60" t="n">
+        <v>22.1978021978022</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>52</v>
+      </c>
+      <c r="B61" t="s">
+        <v>144</v>
+      </c>
+      <c r="C61" t="s">
+        <v>137</v>
+      </c>
+      <c r="D61" t="n">
+        <v>10</v>
+      </c>
+      <c r="E61" t="n">
+        <v>34.3347639484979</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>52</v>
+      </c>
+      <c r="B62" t="s">
+        <v>144</v>
+      </c>
+      <c r="C62" t="s">
+        <v>137</v>
+      </c>
+      <c r="D62" t="n">
+        <v>20</v>
+      </c>
+      <c r="E62" t="n">
+        <v>11.1587982832618</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>52</v>
+      </c>
+      <c r="B63" t="s">
+        <v>144</v>
+      </c>
+      <c r="C63" t="s">
+        <v>140</v>
+      </c>
+      <c r="D63" t="n">
+        <v>10</v>
+      </c>
+      <c r="E63" t="n">
+        <v>46.676970633694</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>52</v>
+      </c>
+      <c r="B64" t="s">
+        <v>144</v>
+      </c>
+      <c r="C64" t="s">
+        <v>140</v>
+      </c>
+      <c r="D64" t="n">
+        <v>20</v>
+      </c>
+      <c r="E64" t="n">
+        <v>21.6383307573416</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>53</v>
+      </c>
+      <c r="B65" t="s">
+        <v>142</v>
+      </c>
+      <c r="C65" t="s">
+        <v>50</v>
+      </c>
+      <c r="D65" t="n">
+        <v>10</v>
+      </c>
+      <c r="E65" t="n">
+        <v>32.0879120879121</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>53</v>
+      </c>
+      <c r="B66" t="s">
+        <v>142</v>
+      </c>
+      <c r="C66" t="s">
+        <v>137</v>
+      </c>
+      <c r="D66" t="n">
+        <v>10</v>
+      </c>
+      <c r="E66" t="n">
+        <v>17.5965665236052</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>53</v>
+      </c>
+      <c r="B67" t="s">
+        <v>142</v>
+      </c>
+      <c r="C67" t="s">
+        <v>140</v>
+      </c>
+      <c r="D67" t="n">
+        <v>10</v>
+      </c>
+      <c r="E67" t="n">
+        <v>11.9010819165379</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>53</v>
+      </c>
+      <c r="B68" t="s">
+        <v>143</v>
+      </c>
+      <c r="C68" t="s">
+        <v>50</v>
+      </c>
+      <c r="D68" t="n">
+        <v>10</v>
+      </c>
+      <c r="E68" t="n">
+        <v>49.2307692307692</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>53</v>
+      </c>
+      <c r="B69" t="s">
+        <v>143</v>
+      </c>
+      <c r="C69" t="s">
+        <v>50</v>
+      </c>
+      <c r="D69" t="n">
+        <v>20</v>
+      </c>
+      <c r="E69" t="n">
+        <v>43.2967032967033</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>53</v>
+      </c>
+      <c r="B70" t="s">
+        <v>143</v>
+      </c>
+      <c r="C70" t="s">
+        <v>50</v>
+      </c>
+      <c r="D70" t="n">
+        <v>40</v>
+      </c>
+      <c r="E70" t="n">
+        <v>38.021978021978</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>53</v>
+      </c>
+      <c r="B71" t="s">
+        <v>143</v>
+      </c>
+      <c r="C71" t="s">
+        <v>50</v>
+      </c>
+      <c r="D71" t="n">
+        <v>80</v>
+      </c>
+      <c r="E71" t="n">
+        <v>28.7912087912088</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>53</v>
+      </c>
+      <c r="B72" t="s">
+        <v>143</v>
+      </c>
+      <c r="C72" t="s">
+        <v>50</v>
+      </c>
+      <c r="D72" t="n">
+        <v>160</v>
+      </c>
+      <c r="E72" t="n">
+        <v>13.6263736263736</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>53</v>
+      </c>
+      <c r="B73" t="s">
+        <v>143</v>
+      </c>
+      <c r="C73" t="s">
+        <v>50</v>
+      </c>
+      <c r="D73" t="n">
+        <v>320</v>
+      </c>
+      <c r="E73" t="n">
+        <v>12.967032967033</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>53</v>
+      </c>
+      <c r="B74" t="s">
+        <v>143</v>
+      </c>
+      <c r="C74" t="s">
+        <v>137</v>
+      </c>
+      <c r="D74" t="n">
+        <v>10</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s">
+        <v>53</v>
+      </c>
+      <c r="B75" t="s">
+        <v>143</v>
+      </c>
+      <c r="C75" t="s">
+        <v>140</v>
+      </c>
+      <c r="D75" t="n">
+        <v>10</v>
+      </c>
+      <c r="E75" t="n">
+        <v>34.1576506955178</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s">
+        <v>53</v>
+      </c>
+      <c r="B76" t="s">
+        <v>144</v>
+      </c>
+      <c r="C76" t="s">
+        <v>50</v>
+      </c>
+      <c r="D76" t="n">
+        <v>10</v>
+      </c>
+      <c r="E76" t="n">
+        <v>82.1978021978022</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s">
+        <v>53</v>
+      </c>
+      <c r="B77" t="s">
+        <v>144</v>
+      </c>
+      <c r="C77" t="s">
+        <v>50</v>
+      </c>
+      <c r="D77" t="n">
+        <v>20</v>
+      </c>
+      <c r="E77" t="n">
+        <v>69.6703296703297</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s">
+        <v>53</v>
+      </c>
+      <c r="B78" t="s">
+        <v>144</v>
+      </c>
+      <c r="C78" t="s">
+        <v>50</v>
+      </c>
+      <c r="D78" t="n">
+        <v>40</v>
+      </c>
+      <c r="E78" t="n">
+        <v>54.5054945054945</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>53</v>
+      </c>
+      <c r="B79" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" t="s">
+        <v>50</v>
+      </c>
+      <c r="D79" t="n">
+        <v>80</v>
+      </c>
+      <c r="E79" t="n">
+        <v>44.6153846153846</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>53</v>
+      </c>
+      <c r="B80" t="s">
+        <v>144</v>
+      </c>
+      <c r="C80" t="s">
+        <v>50</v>
+      </c>
+      <c r="D80" t="n">
+        <v>160</v>
+      </c>
+      <c r="E80" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>53</v>
+      </c>
+      <c r="B81" t="s">
+        <v>144</v>
+      </c>
+      <c r="C81" t="s">
+        <v>50</v>
+      </c>
+      <c r="D81" t="n">
+        <v>320</v>
+      </c>
+      <c r="E81" t="n">
+        <v>34.7252747252747</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s">
+        <v>53</v>
+      </c>
+      <c r="B82" t="s">
+        <v>144</v>
+      </c>
+      <c r="C82" t="s">
+        <v>50</v>
+      </c>
+      <c r="D82" t="n">
+        <v>640</v>
+      </c>
+      <c r="E82" t="n">
+        <v>19.5604395604396</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s">
+        <v>53</v>
+      </c>
+      <c r="B83" t="s">
+        <v>144</v>
+      </c>
+      <c r="C83" t="s">
+        <v>137</v>
+      </c>
+      <c r="D83" t="n">
+        <v>10</v>
+      </c>
+      <c r="E83" t="n">
+        <v>25.3218884120172</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>53</v>
+      </c>
+      <c r="B84" t="s">
+        <v>144</v>
+      </c>
+      <c r="C84" t="s">
+        <v>137</v>
+      </c>
+      <c r="D84" t="n">
+        <v>20</v>
+      </c>
+      <c r="E84" t="n">
+        <v>12.4463519313305</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s">
+        <v>53</v>
+      </c>
+      <c r="B85" t="s">
+        <v>144</v>
+      </c>
+      <c r="C85" t="s">
+        <v>140</v>
+      </c>
+      <c r="D85" t="n">
+        <v>10</v>
+      </c>
+      <c r="E85" t="n">
         <v>25.8114374034003</v>
       </c>
     </row>

</xml_diff>